<commit_message>
formulas-queries-charts SESSION-07: checkpoint 3 — rules from validations; the review surface
</commit_message>
<xml_diff>
--- a/tests/fixtures/workbooks/ooxml/formulas-live.xlsx
+++ b/tests/fixtures/workbooks/ooxml/formulas-live.xlsx
@@ -333,6 +333,11 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" sqref="B2:B6">
+      <formula1>0</formula1>
+    </dataValidation>
+  </dataValidations>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>